<commit_message>
feat(productos): 🚀 Manual del Chef Ejecutivo — LANZAMIENTO (producto 47, 65 €): manual de 96 páginas (20 caps, 52.203 palabras, 42 tablas) + bonus de 34 (12 situaciones resueltas en cocina) + 7 Excel; todos los gates de documentos en verde tras la refutación (27 fixes) y la desduplicación por capítulo (41 pares → 0); landing y email con las páginas medidas; product-prices.ts (47)
Pendiente de John: Payment Link de Stripe (65 €) → env VITE_STRIPE_PAYMENT_LINK_MANUAL_CHEF_EJECUTIVO → sync-payment-links.py. Hasta entonces el CTA enlaza al cajón de compra (#comprar), como toda la familia sin env.

Via: Claude Code

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DhiNDFrceGzPU8tDriiQYd
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/manual-chef-ejecutivo/desarrollo-carta-control-calidad.xlsx
+++ b/astro-site/public/dl/manual-chef-ejecutivo/desarrollo-carta-control-calidad.xlsx
@@ -973,16 +973,16 @@
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>46273</v>
+        <v>46238</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>46280</v>
+        <v>46245</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>46287</v>
+        <v>46256</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>46294</v>
+        <v>46265</v>
       </c>
       <c r="H13" s="6" t="n">
         <v>46301</v>
@@ -999,7 +999,7 @@
       </c>
       <c r="K13" s="12">
         <f>IFERROR(IF(OR($D13="",$C$7=""),"",IF($C$7&lt;$D13,"",$C$7-$D13)),"")</f>
-        <v>16.0</v>
+        <v>51.0</v>
       </c>
       <c r="L13" s="12">
         <f>COUNT($D13:$H13)</f>
@@ -1047,16 +1047,16 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>46275</v>
+        <v>46240</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>46282</v>
+        <v>46247</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>46289</v>
+        <v>46258</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>46296</v>
+        <v>46267</v>
       </c>
       <c r="H14" s="6" t="n">
         <v>46301</v>
@@ -1073,7 +1073,7 @@
       </c>
       <c r="K14" s="12">
         <f>IFERROR(IF(OR($D14="",$C$7=""),"",IF($C$7&lt;$D14,"",$C$7-$D14)),"")</f>
-        <v>14.0</v>
+        <v>49.0</v>
       </c>
       <c r="L14" s="12">
         <f>COUNT($D14:$H14)</f>

</xml_diff>